<commit_message>
lesson16-database sql b2 - ddl
</commit_message>
<xml_diff>
--- a/1. Database Design/Java25 Quyen Phan Database Design.xlsx
+++ b/1. Database Design/Java25 Quyen Phan Database Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798D45C3-5E2B-4357-89FF-B652988A080B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F81AF47-7A7B-4924-B87A-D4083C2179D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -544,6 +544,31 @@
         </r>
       </text>
     </comment>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{81C73AC9-32AB-4DF0-A52C-6090102C1C7C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Có thể trùng tên mặt hàng
+Để =&gt;2 mặt hàng cùng nhưng có màu sắc &amp;| chất liệu khác nhau thì xem như là 2 mặt hàng khác nhau</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B9" authorId="0" shapeId="0" xr:uid="{874A984F-D2B7-4D49-BCF6-0718734568A4}">
       <text>
         <r>
@@ -861,7 +886,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="352">
   <si>
     <t>MatHang</t>
   </si>
@@ -2018,9 +2043,6 @@
     <t>C05_PROVIDER_NAME</t>
   </si>
   <si>
-    <t>C05_PROVIDER_TAX</t>
-  </si>
-  <si>
     <t>C15_AMOUNT</t>
   </si>
   <si>
@@ -2241,13 +2263,16 @@
   </si>
   <si>
     <t>java25_shopping</t>
+  </si>
+  <si>
+    <t>C05_PROVIDER_TAX_PCT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2472,6 +2497,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -2584,7 +2616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2789,6 +2821,12 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4094,46 +4132,46 @@
   <sheetData>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="C2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="D2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="E2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="F2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="G2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="H2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="I2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="J2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="K2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="L2" s="57" t="s">
+        <v>297</v>
+      </c>
+      <c r="M2" s="58" t="s">
         <v>298</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="N2" s="58" t="s">
         <v>298</v>
       </c>
-      <c r="D2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="F2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="G2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="H2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="I2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="J2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="K2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="L2" s="57" t="s">
-        <v>298</v>
-      </c>
-      <c r="M2" s="58" t="s">
-        <v>299</v>
-      </c>
-      <c r="N2" s="58" t="s">
-        <v>299</v>
-      </c>
       <c r="O2" s="57" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -6498,11 +6536,11 @@
         <v>178</v>
       </c>
       <c r="E3" s="60" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F3" s="31"/>
       <c r="G3" s="27" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K3" s="31"/>
       <c r="L3" s="31"/>
@@ -6524,49 +6562,55 @@
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="31"/>
-      <c r="P4" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="Q4" s="31" t="s">
-        <v>298</v>
+      <c r="P4" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="Q4" s="71" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="D5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="E5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="F5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="G5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="H5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="I5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="J5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="K5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="L5" s="31" t="s">
-        <v>298</v>
-      </c>
-      <c r="M5" s="31" t="s">
-        <v>298</v>
+      <c r="B5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="C5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="D5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="E5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="F5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="G5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="H5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="I5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="J5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="K5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="L5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="M5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="N5" s="71" t="s">
+        <v>297</v>
+      </c>
+      <c r="O5" s="71" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6586,37 +6630,37 @@
         <v>274</v>
       </c>
       <c r="G6" s="61" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H6" s="61" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I6" s="61" t="s">
+        <v>299</v>
+      </c>
+      <c r="J6" s="61" t="s">
         <v>300</v>
       </c>
-      <c r="J6" s="61" t="s">
-        <v>301</v>
-      </c>
       <c r="K6" s="61" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="L6" s="61" t="s">
         <v>269</v>
       </c>
       <c r="M6" s="61" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="N6" s="61" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="O6" s="61" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="P6" s="61" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="Q6" s="61" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6636,37 +6680,37 @@
         <v>275</v>
       </c>
       <c r="G7" s="32" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H7" s="32" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I7" s="32" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J7" s="32" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K7" s="32" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="L7" s="32" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="M7" s="60" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="N7" s="60" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="O7" s="60" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="P7" s="32" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="Q7" s="32" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -6686,42 +6730,42 @@
         <v>276</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H8" s="34" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I8" s="35" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J8" s="35" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K8" s="32" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="L8" s="62" t="s">
         <v>270</v>
       </c>
       <c r="M8" s="60" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="N8" s="60" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="O8" s="60" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="P8" s="59" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="Q8" s="59" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="35" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C9" s="35" t="s">
         <v>262</v>
@@ -6733,32 +6777,32 @@
         <v>267</v>
       </c>
       <c r="F9" s="35" t="s">
-        <v>277</v>
+        <v>351</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H9" s="35" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I9" s="59" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J9" s="59" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K9" s="35"/>
       <c r="L9" s="62" t="s">
         <v>271</v>
       </c>
       <c r="M9" s="35" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N9" s="35" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="O9" s="34" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="P9" s="35"/>
       <c r="Q9" s="35"/>
@@ -6766,7 +6810,7 @@
     <row r="10" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31"/>
       <c r="B10" s="35" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C10" s="35"/>
       <c r="D10" s="35"/>
@@ -6775,43 +6819,43 @@
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="35" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H10" s="35"/>
       <c r="I10" s="35" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J10" s="35" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="K10" s="35"/>
       <c r="L10" s="35" t="s">
         <v>272</v>
       </c>
       <c r="M10" s="35" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="N10" s="35"/>
       <c r="O10" s="35" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="P10" s="35"/>
       <c r="Q10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C11" s="35"/>
       <c r="D11" s="35"/>
       <c r="E11" s="35"/>
       <c r="F11" s="35"/>
       <c r="G11" s="35" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H11" s="35"/>
       <c r="I11" s="35" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J11" s="35"/>
       <c r="K11" s="35"/>
@@ -6819,7 +6863,7 @@
         <v>273</v>
       </c>
       <c r="M11" s="35" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="N11" s="35"/>
       <c r="O11" s="35"/>
@@ -6835,11 +6879,11 @@
       <c r="E12" s="35"/>
       <c r="F12" s="35"/>
       <c r="G12" s="35" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H12" s="35"/>
       <c r="I12" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J12" s="35"/>
       <c r="K12" s="35"/>
@@ -6859,11 +6903,11 @@
       <c r="E13" s="35"/>
       <c r="F13" s="35"/>
       <c r="G13" s="34" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H13" s="63"/>
       <c r="I13" s="35" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J13" s="35"/>
       <c r="K13" s="35"/>
@@ -6881,11 +6925,11 @@
       <c r="E14" s="35"/>
       <c r="F14" s="35"/>
       <c r="G14" s="34" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="H14" s="35"/>
       <c r="I14" s="35" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J14" s="35"/>
       <c r="K14" s="35"/>
@@ -7050,14 +7094,14 @@
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="31"/>
-      <c r="B25" s="23" t="s">
-        <v>282</v>
+      <c r="B25" s="72" t="s">
+        <v>281</v>
       </c>
       <c r="C25" s="23"/>
       <c r="D25" s="23"/>
       <c r="E25" s="23"/>
       <c r="G25" s="27" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="K25" s="31"/>
       <c r="L25" s="31"/>
@@ -7066,10 +7110,10 @@
     <row r="26" spans="1:17" s="23" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="31"/>
       <c r="B26" s="54" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K26" s="31"/>
       <c r="L26" s="31"/>
@@ -7077,7 +7121,7 @@
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B27" s="54" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C27" s="23"/>
       <c r="D27" s="23"/>
@@ -7090,7 +7134,7 @@
       <c r="D28" s="23"/>
       <c r="E28" s="23"/>
       <c r="G28" s="27" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K28" s="31"/>
     </row>
@@ -7100,24 +7144,24 @@
       <c r="D29" s="23"/>
       <c r="E29" s="23"/>
       <c r="G29" s="27" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B30" s="56" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C30" s="23"/>
       <c r="D30" s="23"/>
       <c r="E30" s="23"/>
       <c r="G30" s="29" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H30" s="29"/>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B31" s="23" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C31" s="23"/>
       <c r="D31" s="23"/>
@@ -7125,7 +7169,7 @@
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B32" s="23" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C32" s="23"/>
       <c r="D32" s="23"/>
@@ -7149,7 +7193,7 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="66" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C35" s="67"/>
       <c r="D35" s="67"/>
@@ -7159,19 +7203,19 @@
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="29" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="I37" s="29"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="29" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I38" s="29"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="29" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
lesson16-database sql b3 - dml insert delete
</commit_message>
<xml_diff>
--- a/1. Database Design/Java25 Quyen Phan Database Design.xlsx
+++ b/1. Database Design/Java25 Quyen Phan Database Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F81AF47-7A7B-4924-B87A-D4083C2179D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F616EB70-7077-4749-B785-372CA441449D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2813,6 +2813,12 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2821,12 +2827,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5540,10 +5540,10 @@
       <c r="B79" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C79" s="69" t="s">
+      <c r="C79" s="71" t="s">
         <v>178</v>
       </c>
-      <c r="D79" s="70"/>
+      <c r="D79" s="72"/>
       <c r="E79" s="27"/>
       <c r="F79" s="27"/>
       <c r="G79" s="27"/>
@@ -6562,54 +6562,54 @@
       <c r="M4" s="31"/>
       <c r="N4" s="31"/>
       <c r="O4" s="31"/>
-      <c r="P4" s="71" t="s">
+      <c r="P4" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="Q4" s="71" t="s">
+      <c r="Q4" s="68" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="71" t="s">
+      <c r="B5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="D5" s="71" t="s">
+      <c r="D5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="E5" s="71" t="s">
+      <c r="E5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="G5" s="71" t="s">
+      <c r="G5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="H5" s="71" t="s">
+      <c r="H5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="I5" s="71" t="s">
+      <c r="I5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="J5" s="71" t="s">
+      <c r="J5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="K5" s="71" t="s">
+      <c r="K5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="L5" s="71" t="s">
+      <c r="L5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="M5" s="71" t="s">
+      <c r="M5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="N5" s="71" t="s">
+      <c r="N5" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="O5" s="71" t="s">
+      <c r="O5" s="68" t="s">
         <v>297</v>
       </c>
     </row>
@@ -7094,7 +7094,7 @@
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="31"/>
-      <c r="B25" s="72" t="s">
+      <c r="B25" s="69" t="s">
         <v>281</v>
       </c>
       <c r="C25" s="23"/>
@@ -7405,8 +7405,8 @@
     </row>
     <row r="81" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B81" s="31"/>
-      <c r="C81" s="68"/>
-      <c r="D81" s="68"/>
+      <c r="C81" s="70"/>
+      <c r="D81" s="70"/>
     </row>
     <row r="82" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B82" s="50"/>

</xml_diff>

<commit_message>
lesson16-database sql b4 - dml update & select part 1
</commit_message>
<xml_diff>
--- a/1. Database Design/Java25 Quyen Phan Database Design.xlsx
+++ b/1. Database Design/Java25 Quyen Phan Database Design.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\1. Database Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F616EB70-7077-4749-B785-372CA441449D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A63AFD7-78A1-4A98-96F5-DD057377DBC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>